<commit_message>
LIVE_ERP: by Rajsh: 27-07-2026
</commit_message>
<xml_diff>
--- a/public/excel_upload/assets/UPLOAD_tbluser.xlsx
+++ b/public/excel_upload/assets/UPLOAD_tbluser.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\unused\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="8595" windowHeight="7230"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11595"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>user_name</t>
   </si>
@@ -78,19 +83,16 @@
     <t>last_login</t>
   </si>
   <si>
-    <t>qualification</t>
-  </si>
-  <si>
-    <t>pan_no</t>
-  </si>
-  <si>
-    <t>aadhar_no</t>
-  </si>
-  <si>
     <t>joined_date</t>
   </si>
   <si>
-    <t>department_id</t>
+    <t>employee_no</t>
+  </si>
+  <si>
+    <t>pan_card</t>
+  </si>
+  <si>
+    <t>aadhar_card</t>
   </si>
 </sst>
 </file>
@@ -162,6 +164,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -209,7 +214,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -244,7 +249,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -453,15 +458,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -523,19 +547,16 @@
         <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>